<commit_message>
Auto-deploy updates: Wed 09/16/2026 14:47:33.07
</commit_message>
<xml_diff>
--- a/Uploader_Config.xlsx
+++ b/Uploader_Config.xlsx
@@ -1,29 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\NEET Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\NEET Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB6AFC14-7F85-4770-90D4-738772E8C817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA48F0C-7D3E-4122-BEBF-4740047466D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SR ELITE(2025)" sheetId="3" r:id="rId1"/>
     <sheet name="JR ELITE(2025)" sheetId="1" r:id="rId2"/>
     <sheet name="SR ELITE (2026)" sheetId="4" r:id="rId3"/>
     <sheet name="Allowed_Campuses" sheetId="2" r:id="rId4"/>
+    <sheet name="TOP 18" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="11">
   <si>
     <t>STUD_ID</t>
   </si>
@@ -53,6 +67,9 @@
   </si>
   <si>
     <t>SUPER SR ELITE TOP</t>
+  </si>
+  <si>
+    <t>TOP 18</t>
   </si>
 </sst>
 </file>
@@ -3717,4 +3734,112 @@
     <ignoredError sqref="A1:A3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E93AE4D-E3CE-4BBF-8DE6-AC523C7EE6C2}">
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>257403546</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>257404738</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>257403653</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>257427698</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>213309261</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>246556423</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>246555884</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>246555726</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>257407693</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>246556345</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>213307653</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>257420307</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>257400127</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>257403537</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>257409631</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>257402548</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>257405810</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>257406595</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>